<commit_message>
reduced the templates font size
</commit_message>
<xml_diff>
--- a/backend/templates_data/product_import_template.xlsx
+++ b/backend/templates_data/product_import_template.xlsx
@@ -17,13 +17,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
     </font>
   </fonts>
   <fills count="2">
@@ -46,8 +49,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -413,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:F1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -425,59 +429,35 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>name</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>category</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>price</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>cost_price</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>stock_count</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>reorder_point</t>
         </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Coca Cola 500ml</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Beverages</t>
-        </is>
-      </c>
-      <c r="C2" t="n">
-        <v>60</v>
-      </c>
-      <c r="D2" t="n">
-        <v>45</v>
-      </c>
-      <c r="E2" t="n">
-        <v>48</v>
-      </c>
-      <c r="F2" t="n">
-        <v>10</v>
       </c>
     </row>
   </sheetData>

</xml_diff>